<commit_message>
feat: agregar funcionalidad para eliminar asignaturas
- Crear hook useDeleteSubject para manejar eliminación de asignaturas
- Agregar botón de eliminar en subject-detail-page con diálogo de confirmación
- Agregar botón de eliminar en edit-technical-career-page para cada asignatura
- Actualizar SubjectsYearSection para incluir botón de eliminar
- Integrar funcionalidad de eliminación en use-edit-career hook
- Usar soft delete (IsActive = false) en el backend
</commit_message>
<xml_diff>
--- a/alumnos.xlsx
+++ b/alumnos.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">EMAIL</t>
   </si>
@@ -38,6 +38,12 @@
   </si>
   <si>
     <t xml:space="preserve">Alejandro Duarte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tbanchioalumno@itec-elmolino.edu.ar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tomas banchio</t>
   </si>
 </sst>
 </file>
@@ -47,11 +53,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -73,6 +80,14 @@
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -117,12 +132,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -249,41 +272,50 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28.79"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" display="ebottoalumno@itec-elmolino.edu.ar"/>
     <hyperlink ref="A3" r:id="rId2" display="aduartee@itec-elmolino.edu.ar"/>
+    <hyperlink ref="A4" r:id="rId3" display="tbanchioalumno@itec-elmolino.edu.ar"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>